<commit_message>
prepare SCORE data (including 1 directionality fix)
</commit_message>
<xml_diff>
--- a/cos_test1_addition/cos_test_set_phase1_prepared.xlsx
+++ b/cos_test1_addition/cos_test_set_phase1_prepared.xlsx
@@ -1488,7 +1488,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>t-statistic</t>
+          <t>ser_method_t</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>t-statistic</t>
+          <t>ser_method_t</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -6391,7 +6391,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -7432,7 +7432,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -10208,7 +10208,7 @@
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -11204,7 +11204,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -11249,7 +11249,7 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -11596,7 +11596,7 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -12290,7 +12290,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -12637,7 +12637,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
@@ -12984,7 +12984,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -13331,7 +13331,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -13633,7 +13633,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -13678,7 +13678,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
@@ -14327,7 +14327,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
@@ -14372,7 +14372,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -14719,7 +14719,7 @@
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC42" t="inlineStr">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC43" t="inlineStr">
@@ -15413,7 +15413,7 @@
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -15715,7 +15715,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC45" t="inlineStr">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -16107,7 +16107,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -16409,7 +16409,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
@@ -16801,7 +16801,7 @@
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC48" t="inlineStr">
@@ -17103,7 +17103,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -17148,7 +17148,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC49" t="inlineStr">
@@ -17450,7 +17450,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -17495,7 +17495,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC50" t="inlineStr">
@@ -17842,7 +17842,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC51" t="inlineStr">
@@ -18189,7 +18189,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -18491,7 +18491,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -18536,7 +18536,7 @@
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC53" t="inlineStr">
@@ -18838,7 +18838,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -18883,7 +18883,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC54" t="inlineStr">
@@ -19185,7 +19185,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -19230,7 +19230,7 @@
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC55" t="inlineStr">
@@ -19577,7 +19577,7 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC56" t="inlineStr">
@@ -19924,7 +19924,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC57" t="inlineStr">
@@ -20271,7 +20271,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC58" t="inlineStr">
@@ -20573,7 +20573,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -21267,7 +21267,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
@@ -21614,7 +21614,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -21961,7 +21961,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
@@ -22006,7 +22006,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC63" t="inlineStr">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC64" t="inlineStr">
@@ -22655,7 +22655,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
@@ -22700,7 +22700,7 @@
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>t-statistic</t>
+          <t>ser_method_t</t>
         </is>
       </c>
       <c r="AC65" t="inlineStr">
@@ -23002,7 +23002,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
@@ -23047,7 +23047,7 @@
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC66" t="inlineStr">
@@ -26472,7 +26472,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -26517,7 +26517,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC76" t="inlineStr">
@@ -26819,7 +26819,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -26864,7 +26864,7 @@
       </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC77" t="inlineStr">
@@ -27558,7 +27558,7 @@
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC79" t="inlineStr">
@@ -29987,7 +29987,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC86" t="inlineStr">
@@ -30334,7 +30334,7 @@
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC87" t="inlineStr">
@@ -32069,7 +32069,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -33110,7 +33110,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC95" t="inlineStr">
@@ -34498,7 +34498,7 @@
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC99" t="inlineStr">
@@ -35539,7 +35539,7 @@
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC102" t="inlineStr">
@@ -35886,7 +35886,7 @@
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC103" t="inlineStr">
@@ -36927,7 +36927,7 @@
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC106" t="inlineStr">
@@ -37274,7 +37274,7 @@
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>t-statistic</t>
+          <t>ser_method_t</t>
         </is>
       </c>
       <c r="AC107" t="inlineStr">
@@ -37968,7 +37968,7 @@
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC109" t="inlineStr">
@@ -38315,7 +38315,7 @@
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>dz</t>
+          <t>d_sample (dep)</t>
         </is>
       </c>
       <c r="AC110" t="inlineStr">
@@ -38662,7 +38662,7 @@
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC111" t="inlineStr">
@@ -39703,7 +39703,7 @@
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC114" t="inlineStr">
@@ -40050,7 +40050,7 @@
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC115" t="inlineStr">
@@ -41438,7 +41438,7 @@
       </c>
       <c r="AB119" t="inlineStr">
         <is>
-          <t>t-statistic</t>
+          <t>ser_method_t</t>
         </is>
       </c>
       <c r="AC119" t="inlineStr">
@@ -42826,7 +42826,7 @@
       </c>
       <c r="AB123" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC123" t="inlineStr">
@@ -43173,7 +43173,7 @@
       </c>
       <c r="AB124" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC124" t="inlineStr">
@@ -43867,7 +43867,7 @@
       </c>
       <c r="AB126" t="inlineStr">
         <is>
-          <t>test statistic</t>
+          <t>ser_method</t>
         </is>
       </c>
       <c r="AC126" t="inlineStr">

</xml_diff>